<commit_message>
docs(changelog): log the Android port and the four bugs it surfaced
Per CLAUDE.md the changelog is updated as part of a submission, in the same
commit, so the binary .xlsx does not churn on every push.

Nine rows: the port itself, app blocking, and the bugs — Lockbox paying out
without checking the phone, screen-time sync broken for every user on both
platforms, expo-constants four SDKs ahead, the force-update gate that would
have locked out every Android install, SYSTEM_ALERT_WINDOW stripped from
release only, calendar sync refusing to turn on, and the unbuyable Android
paywall. Root cause in Details for each, as the tool's own instructions ask.

Filed as Unreleased: this is on feat/android-port, not main, and nothing has
shipped to a store.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Drift-changelog.xlsx
+++ b/Drift-changelog.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Changes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$123</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -586,7 +586,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-08-28.</t>
+          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-09-11.</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Changes!E2:E114)</f>
+        <f>COUNTA(Changes!E2:E123)</f>
         <v/>
       </c>
     </row>
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$114,A8)</f>
+        <f>COUNTIF(Changes!$C$2:$C$123,A8)</f>
         <v/>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D8)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D8)</f>
         <v/>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$114,G8)</f>
+        <f>COUNTIF(Changes!$G$2:$G$123,G8)</f>
         <v/>
       </c>
     </row>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$114,A9)</f>
+        <f>COUNTIF(Changes!$C$2:$C$123,A9)</f>
         <v/>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D9)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D9)</f>
         <v/>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$114,G9)</f>
+        <f>COUNTIF(Changes!$G$2:$G$123,G9)</f>
         <v/>
       </c>
     </row>
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$114,A10)</f>
+        <f>COUNTIF(Changes!$C$2:$C$123,A10)</f>
         <v/>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D10)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D10)</f>
         <v/>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$114,G10)</f>
+        <f>COUNTIF(Changes!$G$2:$G$123,G10)</f>
         <v/>
       </c>
     </row>
@@ -744,16 +744,16 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$114,A11)</f>
+        <f>COUNTIF(Changes!$C$2:$C$123,A11)</f>
         <v/>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Auth</t>
+          <t>Android</t>
         </is>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D11)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D11)</f>
         <v/>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$114,G11)</f>
+        <f>COUNTIF(Changes!$G$2:$G$123,G11)</f>
         <v/>
       </c>
     </row>
@@ -773,16 +773,16 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$114,A12)</f>
+        <f>COUNTIF(Changes!$C$2:$C$123,A12)</f>
         <v/>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Auth / Sync</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D12)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D12)</f>
         <v/>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="H12" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$114,G12)</f>
+        <f>COUNTIF(Changes!$G$2:$G$123,G12)</f>
         <v/>
       </c>
     </row>
@@ -802,16 +802,16 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$114,A13)</f>
+        <f>COUNTIF(Changes!$C$2:$C$123,A13)</f>
         <v/>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Auth / Sync</t>
         </is>
       </c>
       <c r="E13" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D13)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D13)</f>
         <v/>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -820,7 +820,7 @@
         </is>
       </c>
       <c r="H13" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$114,G13)</f>
+        <f>COUNTIF(Changes!$G$2:$G$123,G13)</f>
         <v/>
       </c>
     </row>
@@ -831,346 +831,390 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$114,A14)</f>
+        <f>COUNTIF(Changes!$C$2:$C$123,A14)</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Billing</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="E14" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D14)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>CI/CD</t>
+          <t>Billing</t>
         </is>
       </c>
       <c r="E15" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D15)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>CI/CD</t>
         </is>
       </c>
       <c r="E16" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D16)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D16)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Challenges</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E17" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D17)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Dependencies</t>
+          <t>Challenges</t>
         </is>
       </c>
       <c r="E18" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D18)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Discoverability</t>
+          <t>Dependencies</t>
         </is>
       </c>
       <c r="E19" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D19)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Drift In</t>
+          <t>Discoverability</t>
         </is>
       </c>
       <c r="E20" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D20)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>Drift In</t>
         </is>
       </c>
       <c r="E21" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D21)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D21)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Growth</t>
+          <t>Family</t>
         </is>
       </c>
       <c r="E22" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D22)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D22)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Interaction</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="E23" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D23)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D23)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Infra</t>
         </is>
       </c>
       <c r="E24" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D24)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D24)</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Interaction</t>
         </is>
       </c>
       <c r="E25" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D25)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>Lockbox</t>
         </is>
       </c>
       <c r="E26" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D26)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="E27" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D27)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E28" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D28)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D28)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="E29" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D29)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D29)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E30" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D30)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D30)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E31" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D31)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D31)</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Scaling</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="E32" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D32)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D32)</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Screen Time</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="E33" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D33)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D33)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="E34" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D34)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D34)</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Siri</t>
+          <t>Scaling</t>
         </is>
       </c>
       <c r="E35" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D35)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D35)</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Sleep Guard</t>
+          <t>Screen Time</t>
         </is>
       </c>
       <c r="E36" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D36)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D36)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Tasks</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="E37" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D37)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D37)</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>Siri</t>
         </is>
       </c>
       <c r="E38" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D38)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D38)</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Tour</t>
+          <t>Sleep Guard</t>
         </is>
       </c>
       <c r="E39" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D39)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D39)</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Tasks</t>
         </is>
       </c>
       <c r="E40" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D40)</f>
+        <f>COUNTIF(Changes!$D$2:$D$123,D40)</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="D41" s="7" t="inlineStr">
         <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="E41" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$123,D41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Tour</t>
+        </is>
+      </c>
+      <c r="E42" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$123,D42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E43" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$123,D43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Updates</t>
+        </is>
+      </c>
+      <c r="E44" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$123,D44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="D45" s="7" t="inlineStr">
+        <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="E41" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$114,D41)</f>
+      <c r="E45" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$123,D45)</f>
         <v/>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="13" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="13" t="inlineStr">
         <is>
           <t>• 1.1.4 is the last version submitted to the App Store. Everything marked Unreleased is on main but not shipped.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="13" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="13" t="inlineStr">
         <is>
           <t>• "Needs" says what a change requires beyond a normal JS reload: a native rebuild, an edge-function deploy, or SQL run in Supabase.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="13" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
         <is>
           <t>• Native-build items are currently blocked on Apple Developer account access, so they are not device-tested.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="13" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="13" t="inlineStr">
         <is>
           <t>• Counts on this sheet are formulas over the Changes tab — they update if you edit, add or delete rows there.</t>
         </is>
@@ -1187,7 +1231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H114"/>
+  <dimension ref="A1:H123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5980,8 +6024,386 @@
         </is>
       </c>
     </row>
+    <row r="115" ht="40" customHeight="1">
+      <c r="A115" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B115" s="16" t="inlineStr">
+        <is>
+          <t>dcaf805</t>
+        </is>
+      </c>
+      <c r="C115" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D115" s="15" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="E115" s="18" t="inlineStr">
+        <is>
+          <t>Drift runs on Android</t>
+        </is>
+      </c>
+      <c r="F115" s="18" t="inlineStr">
+        <is>
+          <t>Native project generated and committed alongside ios/. All four Android icons are derived from the single iOS app icon by tools/build-android-icons.js so there is one source of truth - the notification icon has to be a white silhouette because Android discards colour and keeps only the alpha channel, and a coloured one renders as a white blob. Four notification channels replace the single bucket expo-notifications would otherwise invent, so muting the daily streak nudge no longer also mutes a lockbox breach warning.</t>
+        </is>
+      </c>
+      <c r="G115" s="25" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H115" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="40" customHeight="1">
+      <c r="A116" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B116" s="16" t="inlineStr">
+        <is>
+          <t>afe45b5</t>
+        </is>
+      </c>
+      <c r="C116" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D116" s="15" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="E116" s="18" t="inlineStr">
+        <is>
+          <t>App blocking on Android, without Family Controls</t>
+        </is>
+      </c>
+      <c r="F116" s="18" t="inlineStr">
+        <is>
+          <t>Android exposes no API for one app to shield another, so Drift does it itself: a foreground service polling UsageStatsManager at 1Hz, an optional AccessibilityService for instant detection, and a full ShieldActivity - an activity rather than a floating overlay, so the blocked app is paused by the OS instead of left playing underneath. Built as a local Expo module so `expo prebuild --clean` cannot wipe it. The JS interface mirrors iOS ScreenTimeModule exactly, so Drift In, blocked hours and the balance reconcile drive it through calls they already made and no screen needed rewriting. Verified on device, including after a reboot with Drift never opened.</t>
+        </is>
+      </c>
+      <c r="G116" s="25" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H116" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="40" customHeight="1">
+      <c r="A117" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B117" s="16" t="inlineStr">
+        <is>
+          <t>ef7d882</t>
+        </is>
+      </c>
+      <c r="C117" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D117" s="15" t="inlineStr">
+        <is>
+          <t>Lockbox</t>
+        </is>
+      </c>
+      <c r="E117" s="18" t="inlineStr">
+        <is>
+          <t>Lockbox handed out screen time without ever checking the phone (Android)</t>
+        </is>
+      </c>
+      <c r="F117" s="18" t="inlineStr">
+        <is>
+          <t>startMonitoring() threw "unavailable" on Android and every call site swallowed it, and onStateChange() returned a no-op - so markDisturbed(), the only route to forfeiting a session, could never fire. Every session ran to settle("completed") and awarded the full reward whether or not the phone went in the box: start a 90-minute session, use the phone throughout, collect 45 minutes. Fixed by porting the iOS motion sensing to SensorManager with the constants copied rather than re-tuned. One real difference: both platforms point z out through the screen but disagree on the sign, so Android tests gravity.z &gt; +0.8g for face-up where iOS tests &lt; -0.8.</t>
+        </is>
+      </c>
+      <c r="G117" s="25" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H117" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="40" customHeight="1">
+      <c r="A118" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B118" s="16" t="inlineStr">
+        <is>
+          <t>0e939db</t>
+        </is>
+      </c>
+      <c r="C118" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D118" s="15" t="inlineStr">
+        <is>
+          <t>Screen Time</t>
+        </is>
+      </c>
+      <c r="E118" s="18" t="inlineStr">
+        <is>
+          <t>Screen-time sync had been failing for every user on both platforms</t>
+        </is>
+      </c>
+      <c r="F118" s="18" t="inlineStr">
+        <is>
+          <t>syncScreenTime warned 'record new has no field updated_at' on every call. schema_v7 declared the column inside `create table IF NOT EXISTS public.screen_time`, but the table already existed from schema_v2, so the whole CREATE was skipped and the column never landed; spent_minutes survived only because it got its own explicit ALTER afterwards. The trigger referencing it was created unconditionally and has thrown ever since. Because the upsert conflicts on (user_id, date), the first write each day INSERTed and succeeded while every later write UPDATEd and failed - which is why the friends leaderboard showed stale screen time rather than none. Confirmed with a PostgREST probe (42703 before, 200 after) rather than from the push output.</t>
+        </is>
+      </c>
+      <c r="G118" s="25" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H118" s="22" t="inlineStr">
+        <is>
+          <t>SQL migration</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="40" customHeight="1">
+      <c r="A119" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B119" s="16" t="inlineStr">
+        <is>
+          <t>4042b4c</t>
+        </is>
+      </c>
+      <c r="C119" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D119" s="15" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E119" s="18" t="inlineStr">
+        <is>
+          <t>expo-constants was pinned four SDKs ahead of the project</t>
+        </is>
+      </c>
+      <c r="F119" s="18" t="inlineStr">
+        <is>
+          <t>package.json carried expo-constants ^57.0.8 against Expo SDK 54, which expects ~18.0.14 - the only expo-* dependency using a caret. iOS tolerated it; Android would not compile at all, because that version calls expo.modules.kotlin.services.ServiceInterface, which does not exist in SDK 54 expo-modules-core. react-native-svg was also behind and aborted the process during Fabric component registration before a single frame rendered.</t>
+        </is>
+      </c>
+      <c r="G119" s="25" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H119" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="40" customHeight="1">
+      <c r="A120" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B120" s="16" t="inlineStr">
+        <is>
+          <t>82407e9</t>
+        </is>
+      </c>
+      <c r="C120" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D120" s="15" t="inlineStr">
+        <is>
+          <t>Updates</t>
+        </is>
+      </c>
+      <c r="E120" s="18" t="inlineStr">
+        <is>
+          <t>The force-update gate would have locked out every Android install</t>
+        </is>
+      </c>
+      <c r="F120" s="18" t="inlineStr">
+        <is>
+          <t>Check 2 read app_config.min_ios_version with no platform guard, while checks 1 and 3 were iOS-gated. Setting that key for an iOS hotfix would have caught every Android install too and held it behind ForceUpdateModal - which has no dismiss - pointed at an App Store URL it cannot install from. The same class of lockout as 2026-07-29, arriving from a config row instead of a stale app.json. All four keys are now per-store, and the Android ones do not exist yet, so Android is inert by default.</t>
+        </is>
+      </c>
+      <c r="G120" s="25" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H120" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="40" customHeight="1">
+      <c r="A121" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B121" s="16" t="inlineStr">
+        <is>
+          <t>afe45b5</t>
+        </is>
+      </c>
+      <c r="C121" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D121" s="15" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="E121" s="18" t="inlineStr">
+        <is>
+          <t>Blocking would have worked in every dev build and died in production</t>
+        </is>
+      </c>
+      <c r="F121" s="18" t="inlineStr">
+        <is>
+          <t>SYSTEM_ALERT_WINDOW sat in blockedPermissions from when it looked unused. React Native declares it independently in the debug manifest for the dev overlay, so it was present in every debug build and stripped from release - canDrawOverlays() would have returned false forever, the shield would never have launched, and the permission would not even have appeared in Settings for the user to grant. Caught by diffing the merged debug and release manifests, which is now worth doing before any submission.</t>
+        </is>
+      </c>
+      <c r="G121" s="25" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H121" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="40" customHeight="1">
+      <c r="A122" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B122" s="16" t="inlineStr">
+        <is>
+          <t>603c608</t>
+        </is>
+      </c>
+      <c r="C122" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D122" s="15" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="E122" s="18" t="inlineStr">
+        <is>
+          <t>Calendar sync silently refused to turn on</t>
+        </is>
+      </c>
+      <c r="F122" s="18" t="inlineStr">
+        <is>
+          <t>The toggle flipped on and immediately back off, with no dialog and no error. expo-calendar requests READ_CALENDAR and WRITE_CALENDAR together and gates on hasGrantedPermissions(READ, WRITE) - both - but WRITE was in blockedPermissions, so it could never be granted and toggleCalendar() reverted itself. Drift still never writes to a calendar; the permission is held only because the expo-calendar gate demands it. WRITE_CONTACTS stays blocked, because expo-contacts checks isPermissionPresentInManifest first and asks for READ alone when it is absent.</t>
+        </is>
+      </c>
+      <c r="G122" s="25" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H122" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="40" customHeight="1">
+      <c r="A123" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B123" s="16" t="inlineStr">
+        <is>
+          <t>dcaf805</t>
+        </is>
+      </c>
+      <c r="C123" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D123" s="15" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="E123" s="18" t="inlineStr">
+        <is>
+          <t>Android users would have hit a paywall they could not buy through</t>
+        </is>
+      </c>
+      <c r="F123" s="18" t="inlineStr">
+        <is>
+          <t>RevenueCat issues one public SDK key per store and they are not interchangeable, but every non-iOS caller got "not_ios" and failed closed. Now platform-selected via EXPO_PUBLIC_RC_ANDROID_KEY, deliberately with no hardcoded fallback: the 2026-08-28 note in that file records a stale hardcoded key outliving its app and shipping silently in every build, because a wrong key fails exactly like a missing one except a missing one says so.</t>
+        </is>
+      </c>
+      <c r="G123" s="25" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H123" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H114"/>
+  <autoFilter ref="A1:H123"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(release): 1.1.8, changelog updated
Ships the Johns Hopkins pilot tracking: participant IDs at code
redemption, blocked-app and screen-view events, the Screen Time prompt
answer, and the shield's app-switcher fix.

Version bumped in app.json, package.json and MARKETING_VERSION together,
since the force-update gate reads app.json and locks out every install
when they disagree. Xcode Cloud assigns the build number.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Drift-changelog.xlsx
+++ b/Drift-changelog.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$133</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -586,7 +586,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-09-11.</t>
+          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-09-19.</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Changes!E2:E127)</f>
+        <f>COUNTA(Changes!E2:E133)</f>
         <v/>
       </c>
     </row>
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$127,A8)</f>
+        <f>COUNTIF(Changes!$C$2:$C$133,A8)</f>
         <v/>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D8)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D8)</f>
         <v/>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$127,G8)</f>
+        <f>COUNTIF(Changes!$G$2:$G$133,G8)</f>
         <v/>
       </c>
     </row>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$127,A9)</f>
+        <f>COUNTIF(Changes!$C$2:$C$133,A9)</f>
         <v/>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D9)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D9)</f>
         <v/>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$127,G9)</f>
+        <f>COUNTIF(Changes!$G$2:$G$133,G9)</f>
         <v/>
       </c>
     </row>
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$127,A10)</f>
+        <f>COUNTIF(Changes!$C$2:$C$133,A10)</f>
         <v/>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D10)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D10)</f>
         <v/>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$127,G10)</f>
+        <f>COUNTIF(Changes!$G$2:$G$133,G10)</f>
         <v/>
       </c>
     </row>
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$127,A11)</f>
+        <f>COUNTIF(Changes!$C$2:$C$133,A11)</f>
         <v/>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D11)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D11)</f>
         <v/>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$127,G11)</f>
+        <f>COUNTIF(Changes!$G$2:$G$133,G11)</f>
         <v/>
       </c>
     </row>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$127,A12)</f>
+        <f>COUNTIF(Changes!$C$2:$C$133,A12)</f>
         <v/>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D12)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D12)</f>
         <v/>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="H12" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$127,G12)</f>
+        <f>COUNTIF(Changes!$G$2:$G$133,G12)</f>
         <v/>
       </c>
     </row>
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$127,A13)</f>
+        <f>COUNTIF(Changes!$C$2:$C$133,A13)</f>
         <v/>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -811,16 +811,16 @@
         </is>
       </c>
       <c r="E13" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D13)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D13)</f>
         <v/>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Unreleased</t>
+          <t>1.1.8</t>
         </is>
       </c>
       <c r="H13" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$127,G13)</f>
+        <f>COUNTIF(Changes!$G$2:$G$133,G13)</f>
         <v/>
       </c>
     </row>
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$127,A14)</f>
+        <f>COUNTIF(Changes!$C$2:$C$133,A14)</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -840,7 +840,16 @@
         </is>
       </c>
       <c r="E14" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D14)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H14" s="7">
+        <f>COUNTIF(Changes!$G$2:$G$133,G14)</f>
         <v/>
       </c>
     </row>
@@ -851,7 +860,7 @@
         </is>
       </c>
       <c r="E15" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D15)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D15)</f>
         <v/>
       </c>
     </row>
@@ -862,7 +871,7 @@
         </is>
       </c>
       <c r="E16" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D16)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D16)</f>
         <v/>
       </c>
     </row>
@@ -873,7 +882,7 @@
         </is>
       </c>
       <c r="E17" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D17)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D17)</f>
         <v/>
       </c>
     </row>
@@ -884,370 +893,381 @@
         </is>
       </c>
       <c r="E18" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D18)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Dependencies</t>
+          <t>Cohort codes</t>
         </is>
       </c>
       <c r="E19" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D19)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Discoverability</t>
+          <t>Dependencies</t>
         </is>
       </c>
       <c r="E20" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D20)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Drift In</t>
+          <t>Discoverability</t>
         </is>
       </c>
       <c r="E21" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D21)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D21)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>Drift In</t>
         </is>
       </c>
       <c r="E22" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D22)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D22)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>Entitlement</t>
         </is>
       </c>
       <c r="E23" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D23)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D23)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Force update</t>
+          <t>Family</t>
         </is>
       </c>
       <c r="E24" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D24)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D24)</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Growth</t>
+          <t>Force update</t>
         </is>
       </c>
       <c r="E25" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D25)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Interaction</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="E26" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D26)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Lockbox</t>
+          <t>Interaction</t>
         </is>
       </c>
       <c r="E27" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D27)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Lockbox</t>
         </is>
       </c>
       <c r="E28" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D28)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D28)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="E29" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D29)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D29)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E30" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D30)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D30)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="E31" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D31)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D31)</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Paywall</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E32" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D32)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D32)</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Paywall</t>
         </is>
       </c>
       <c r="E33" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D33)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D33)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E34" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D34)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D34)</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="E35" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D35)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D35)</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="E36" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D36)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D36)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Reviews</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="E37" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D37)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D37)</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Scaling</t>
+          <t>Reviews</t>
         </is>
       </c>
       <c r="E38" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D38)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D38)</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Screen Time</t>
+          <t>Scaling</t>
         </is>
       </c>
       <c r="E39" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D39)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D39)</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Screen Time</t>
         </is>
       </c>
       <c r="E40" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D40)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D40)</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Siri</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="E41" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D41)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D41)</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Sleep Guard</t>
+          <t>Siri</t>
         </is>
       </c>
       <c r="E42" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D42)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D42)</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Social</t>
+          <t>Sleep Guard</t>
         </is>
       </c>
       <c r="E43" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D43)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D43)</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Tasks</t>
+          <t>Social</t>
         </is>
       </c>
       <c r="E44" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D44)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D44)</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>Tasks</t>
         </is>
       </c>
       <c r="E45" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D45)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D45)</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Tour</t>
+          <t>Theme</t>
         </is>
       </c>
       <c r="E46" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D46)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D46)</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Tour</t>
         </is>
       </c>
       <c r="E47" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D47)</f>
+        <f>COUNTIF(Changes!$D$2:$D$133,D47)</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="D48" s="7" t="inlineStr">
         <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E48" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$133,D48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="D49" s="7" t="inlineStr">
+        <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="E48" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$127,D48)</f>
+      <c r="E49" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$133,D49)</f>
         <v/>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="13" t="inlineStr">
-        <is>
-          <t>• 1.1.4 is the last version submitted to the App Store. Everything marked Unreleased is on main but not shipped.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>• "Needs" says what a change requires beyond a normal JS reload: a native rebuild, an edge-function deploy, or SQL run in Supabase.</t>
+          <t>• 1.1.4 is the last version submitted to the App Store. Everything marked Unreleased is on main but not shipped.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>• Native-build items are currently blocked on Apple Developer account access, so they are not device-tested.</t>
+          <t>• "Needs" says what a change requires beyond a normal JS reload: a native rebuild, an edge-function deploy, or SQL run in Supabase.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>• Native-build items are currently blocked on Apple Developer account access, so they are not device-tested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="13" t="inlineStr">
         <is>
           <t>• Counts on this sheet are formulas over the Changes tab — they update if you edit, add or delete rows there.</t>
         </is>
@@ -1264,7 +1284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H127"/>
+  <dimension ref="A1:H133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -6603,8 +6623,260 @@
         </is>
       </c>
     </row>
+    <row r="128" ht="40" customHeight="1">
+      <c r="A128" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B128" s="16" t="inlineStr">
+        <is>
+          <t>81d40da</t>
+        </is>
+      </c>
+      <c r="C128" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D128" s="15" t="inlineStr">
+        <is>
+          <t>Cohort codes</t>
+        </is>
+      </c>
+      <c r="E128" s="18" t="inlineStr">
+        <is>
+          <t>Study participants enter their participant ID when they redeem a code</t>
+        </is>
+      </c>
+      <c r="F128" s="18" t="inlineStr">
+        <is>
+          <t>The Johns Hopkins pilot reports per participant keyed on the study's own IDs, never names or emails. A code can carry participant_id_format; when set, redemption asks for the ID, checks the format, refuses one already used on that code, and stores it uppercased so 'jhu-007' and 'JHU-007' are one person. No seat is spent until the ID is accepted, and codes without a format are unchanged. cohort_participants(cohort) returns the funnel by ID only.</t>
+        </is>
+      </c>
+      <c r="G128" s="16" t="inlineStr">
+        <is>
+          <t>1.1.8</t>
+        </is>
+      </c>
+      <c r="H128" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="40" customHeight="1">
+      <c r="A129" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B129" s="16" t="inlineStr">
+        <is>
+          <t>5ef1f3a</t>
+        </is>
+      </c>
+      <c r="C129" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D129" s="15" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="E129" s="18" t="inlineStr">
+        <is>
+          <t>Blocking an app is finally recorded on the server</t>
+        </is>
+      </c>
+      <c r="F129" s="18" t="inlineStr">
+        <is>
+          <t>Apple's picker keeps the selection on the device and nothing wrote the blocked_apps table, so a user who blocked apps was indistinguishable from one who never did - the 'activated' step of the pilot funnel. Now logs counts only (apps, categories, web domains), never names or tokens.</t>
+        </is>
+      </c>
+      <c r="G129" s="16" t="inlineStr">
+        <is>
+          <t>1.1.8</t>
+        </is>
+      </c>
+      <c r="H129" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="40" customHeight="1">
+      <c r="A130" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B130" s="16" t="inlineStr">
+        <is>
+          <t>affed23</t>
+        </is>
+      </c>
+      <c r="C130" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D130" s="15" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="E130" s="18" t="inlineStr">
+        <is>
+          <t>Screen views recorded per tab</t>
+        </is>
+      </c>
+      <c r="F130" s="18" t="inlineStr">
+        <is>
+          <t>trackScreen existed since analytics landed but nothing ever called it, so which features people use was invisible. Fires once per tab change.</t>
+        </is>
+      </c>
+      <c r="G130" s="16" t="inlineStr">
+        <is>
+          <t>1.1.8</t>
+        </is>
+      </c>
+      <c r="H130" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="40" customHeight="1">
+      <c r="A131" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B131" s="16" t="inlineStr">
+        <is>
+          <t>c006b06</t>
+        </is>
+      </c>
+      <c r="C131" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D131" s="15" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="E131" s="18" t="inlineStr">
+        <is>
+          <t>Failed event uploads were silently discarded</t>
+        </is>
+      </c>
+      <c r="F131" s="18" t="inlineStr">
+        <is>
+          <t>supabase-js returns insert errors rather than throwing them, so the bare try/catch around the flush hid every rejected batch; a day with no events read exactly like a day with no users. Dev builds now log the failure. Found while verifying the pilot funnel on device.</t>
+        </is>
+      </c>
+      <c r="G131" s="16" t="inlineStr">
+        <is>
+          <t>1.1.8</t>
+        </is>
+      </c>
+      <c r="H131" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="40" customHeight="1">
+      <c r="A132" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B132" s="16" t="inlineStr">
+        <is>
+          <t>7aaa9ee</t>
+        </is>
+      </c>
+      <c r="C132" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D132" s="15" t="inlineStr">
+        <is>
+          <t>Screen Time</t>
+        </is>
+      </c>
+      <c r="E132" s="18" t="inlineStr">
+        <is>
+          <t>White border around the block screen in the app switcher</t>
+        </is>
+      </c>
+      <c r="F132" s="18" t="inlineStr">
+        <is>
+          <t>The shield drew an opaque colour with no background blur style, so the blocked app's own window showed through as a white frame in the switcher snapshot, on every blocked app regardless of theme. A material makes iOS composite the shield across the whole snapshot; the opaque ground keeps the shield itself solid in use. Verified on device.</t>
+        </is>
+      </c>
+      <c r="G132" s="16" t="inlineStr">
+        <is>
+          <t>1.1.8</t>
+        </is>
+      </c>
+      <c r="H132" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="40" customHeight="1">
+      <c r="A133" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B133" s="16" t="inlineStr">
+        <is>
+          <t>c79f41c</t>
+        </is>
+      </c>
+      <c r="C133" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D133" s="15" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="E133" s="18" t="inlineStr">
+        <is>
+          <t>The answer to Apple's Screen Time prompt is recorded</t>
+        </is>
+      </c>
+      <c r="F133" s="18" t="inlineStr">
+        <is>
+          <t>Nothing works without that permission and the answer was used then thrown away, so a signup that never blocked anything looked the same as one that refused. Wrapped at the bridge layer so every path that asks is covered.</t>
+        </is>
+      </c>
+      <c r="G133" s="16" t="inlineStr">
+        <is>
+          <t>1.1.8</t>
+        </is>
+      </c>
+      <c r="H133" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H127"/>
+  <autoFilter ref="A1:H133"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(release): keep this release as 1.1.7, not 1.1.8
1.1.7 was pulled back from review and never reached the App Store, which
still serves 1.1.6. Reusing the number keeps users from skipping a
version that only ever existed in our own records. App Store Connect
only requires the version and build number pair to be unique, and Xcode
Cloud assigns a fresh build number.

Reverts the bump in 165e3d8 and relabels its six changelog rows.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Drift-changelog.xlsx
+++ b/Drift-changelog.xlsx
@@ -816,7 +816,7 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>1.1.8</t>
+          <t>Unreleased</t>
         </is>
       </c>
       <c r="H13" s="7">
@@ -841,15 +841,6 @@
       </c>
       <c r="E14" s="7">
         <f>COUNTIF(Changes!$D$2:$D$133,D14)</f>
-        <v/>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>Unreleased</t>
-        </is>
-      </c>
-      <c r="H14" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$133,G14)</f>
         <v/>
       </c>
     </row>
@@ -6656,7 +6647,7 @@
       </c>
       <c r="G128" s="16" t="inlineStr">
         <is>
-          <t>1.1.8</t>
+          <t>1.1.7</t>
         </is>
       </c>
       <c r="H128" s="16" t="inlineStr">
@@ -6698,7 +6689,7 @@
       </c>
       <c r="G129" s="16" t="inlineStr">
         <is>
-          <t>1.1.8</t>
+          <t>1.1.7</t>
         </is>
       </c>
       <c r="H129" s="16" t="inlineStr">
@@ -6740,7 +6731,7 @@
       </c>
       <c r="G130" s="16" t="inlineStr">
         <is>
-          <t>1.1.8</t>
+          <t>1.1.7</t>
         </is>
       </c>
       <c r="H130" s="16" t="inlineStr">
@@ -6782,7 +6773,7 @@
       </c>
       <c r="G131" s="16" t="inlineStr">
         <is>
-          <t>1.1.8</t>
+          <t>1.1.7</t>
         </is>
       </c>
       <c r="H131" s="16" t="inlineStr">
@@ -6824,7 +6815,7 @@
       </c>
       <c r="G132" s="16" t="inlineStr">
         <is>
-          <t>1.1.8</t>
+          <t>1.1.7</t>
         </is>
       </c>
       <c r="H132" s="16" t="inlineStr">
@@ -6866,7 +6857,7 @@
       </c>
       <c r="G133" s="16" t="inlineStr">
         <is>
-          <t>1.1.8</t>
+          <t>1.1.7</t>
         </is>
       </c>
       <c r="H133" s="16" t="inlineStr">

</xml_diff>

<commit_message>
chore(changelog): 1.1.8 review fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Drift-changelog.xlsx
+++ b/Drift-changelog.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$145</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$150</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-09-29.</t>
+          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-10-01.</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Changes!E2:E145)</f>
+        <f>COUNTA(Changes!E2:E150)</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$145,A8)</f>
+        <f>COUNTIF(Changes!$C$2:$C$150,A8)</f>
         <v/>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D8)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D8)</f>
         <v/>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$145,G8)</f>
+        <f>COUNTIF(Changes!$G$2:$G$150,G8)</f>
         <v/>
       </c>
     </row>
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$145,A9)</f>
+        <f>COUNTIF(Changes!$C$2:$C$150,A9)</f>
         <v/>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D9)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D9)</f>
         <v/>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$145,G9)</f>
+        <f>COUNTIF(Changes!$G$2:$G$150,G9)</f>
         <v/>
       </c>
     </row>
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$145,A10)</f>
+        <f>COUNTIF(Changes!$C$2:$C$150,A10)</f>
         <v/>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D10)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D10)</f>
         <v/>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$145,G10)</f>
+        <f>COUNTIF(Changes!$G$2:$G$150,G10)</f>
         <v/>
       </c>
     </row>
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$145,A11)</f>
+        <f>COUNTIF(Changes!$C$2:$C$150,A11)</f>
         <v/>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D11)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D11)</f>
         <v/>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$145,G11)</f>
+        <f>COUNTIF(Changes!$G$2:$G$150,G11)</f>
         <v/>
       </c>
     </row>
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$145,A12)</f>
+        <f>COUNTIF(Changes!$C$2:$C$150,A12)</f>
         <v/>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D12)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D12)</f>
         <v/>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="H12" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$145,G12)</f>
+        <f>COUNTIF(Changes!$G$2:$G$150,G12)</f>
         <v/>
       </c>
     </row>
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$145,A13)</f>
+        <f>COUNTIF(Changes!$C$2:$C$150,A13)</f>
         <v/>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="E13" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D13)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D13)</f>
         <v/>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="H13" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$145,G13)</f>
+        <f>COUNTIF(Changes!$G$2:$G$150,G13)</f>
         <v/>
       </c>
     </row>
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$145,A14)</f>
+        <f>COUNTIF(Changes!$C$2:$C$150,A14)</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="E14" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D14)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D14)</f>
         <v/>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="H14" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$145,G14)</f>
+        <f>COUNTIF(Changes!$G$2:$G$150,G14)</f>
         <v/>
       </c>
     </row>
@@ -852,7 +852,7 @@
         </is>
       </c>
       <c r="E15" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D15)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D15)</f>
         <v/>
       </c>
     </row>
@@ -863,7 +863,7 @@
         </is>
       </c>
       <c r="E16" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D16)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D16)</f>
         <v/>
       </c>
     </row>
@@ -874,7 +874,7 @@
         </is>
       </c>
       <c r="E17" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D17)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D17)</f>
         <v/>
       </c>
     </row>
@@ -885,414 +885,425 @@
         </is>
       </c>
       <c r="E18" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D18)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Cohort codes</t>
+          <t>Codes</t>
         </is>
       </c>
       <c r="E19" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D19)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Dependencies</t>
+          <t>Cohort codes</t>
         </is>
       </c>
       <c r="E20" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D20)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Dev</t>
+          <t>Dependencies</t>
         </is>
       </c>
       <c r="E21" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D21)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D21)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Discoverability</t>
+          <t>Dev</t>
         </is>
       </c>
       <c r="E22" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D22)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D22)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Drift In</t>
+          <t>Discoverability</t>
         </is>
       </c>
       <c r="E23" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D23)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D23)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>Drift In</t>
         </is>
       </c>
       <c r="E24" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D24)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D24)</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>Entitlement</t>
         </is>
       </c>
       <c r="E25" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D25)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Force update</t>
+          <t>Family</t>
         </is>
       </c>
       <c r="E26" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D26)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Growth</t>
+          <t>Force update</t>
         </is>
       </c>
       <c r="E27" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D27)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Interaction</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="E28" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D28)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D28)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Lab</t>
+          <t>Interaction</t>
         </is>
       </c>
       <c r="E29" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D29)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D29)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Live Activity</t>
+          <t>Lab</t>
         </is>
       </c>
       <c r="E30" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D30)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D30)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Lockbox</t>
+          <t>Live Activity</t>
         </is>
       </c>
       <c r="E31" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D31)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D31)</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Lockbox</t>
         </is>
       </c>
       <c r="E32" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D32)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D32)</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="E33" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D33)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D33)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E34" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D34)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D34)</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="E35" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D35)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D35)</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Paywall</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E36" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D36)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D36)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Paywall</t>
         </is>
       </c>
       <c r="E37" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D37)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D37)</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E38" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D38)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D38)</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="E39" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D39)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D39)</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="E40" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D40)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D40)</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Reviews</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="E41" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D41)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D41)</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Scaling</t>
+          <t>Reviews</t>
         </is>
       </c>
       <c r="E42" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D42)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D42)</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Screen Time</t>
+          <t>Scaling</t>
         </is>
       </c>
       <c r="E43" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D43)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D43)</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Screen Time</t>
         </is>
       </c>
       <c r="E44" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D44)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D44)</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Siri</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="E45" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D45)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D45)</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Sleep Guard</t>
+          <t>Siri</t>
         </is>
       </c>
       <c r="E46" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D46)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D46)</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Social</t>
+          <t>Sleep Guard</t>
         </is>
       </c>
       <c r="E47" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D47)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D47)</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Tasks</t>
+          <t>Social</t>
         </is>
       </c>
       <c r="E48" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D48)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D48)</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>Tasks</t>
         </is>
       </c>
       <c r="E49" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D49)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D49)</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Tour</t>
+          <t>Theme</t>
         </is>
       </c>
       <c r="E50" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D50)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D50)</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Tour</t>
         </is>
       </c>
       <c r="E51" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D51)</f>
+        <f>COUNTIF(Changes!$D$2:$D$150,D51)</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="D52" s="7" t="inlineStr">
         <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E52" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$150,D52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="D53" s="7" t="inlineStr">
+        <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="E52" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$145,D52)</f>
+      <c r="E53" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$150,D53)</f>
         <v/>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="13" t="inlineStr">
-        <is>
-          <t>• 1.1.8 is the last version submitted to the App Store. Everything marked Unreleased is on main but not shipped.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>• "Needs" says what a change requires beyond a normal JS reload: a native rebuild, an edge-function deploy, or SQL run in Supabase.</t>
+          <t>• 1.1.8 is the last version submitted to the App Store. Everything marked Unreleased is on main but not shipped.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>• Native-build items are currently blocked on Apple Developer account access, so they are not device-tested.</t>
+          <t>• "Needs" says what a change requires beyond a normal JS reload: a native rebuild, an edge-function deploy, or SQL run in Supabase.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>• Native-build items are currently blocked on Apple Developer account access, so they are not device-tested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
         <is>
           <t>• Counts on this sheet are formulas over the Changes tab — they update if you edit, add or delete rows there.</t>
         </is>
@@ -1309,7 +1320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H145"/>
+  <dimension ref="A1:H150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7404,8 +7415,218 @@
         </is>
       </c>
     </row>
+    <row r="146" ht="40" customHeight="1">
+      <c r="A146" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B146" s="16" t="inlineStr">
+        <is>
+          <t>56843dd</t>
+        </is>
+      </c>
+      <c r="C146" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D146" s="15" t="inlineStr">
+        <is>
+          <t>Lockbox</t>
+        </is>
+      </c>
+      <c r="E146" s="18" t="inlineStr">
+        <is>
+          <t>A finished Lockbox session could pay out twice</t>
+        </is>
+      </c>
+      <c r="F146" s="18" t="inlineStr">
+        <is>
+          <t>finishSession read the session, appended history, then cleared it, with nothing stopping a second caller in between. The countdown, the grace ticker and the End button can all settle at once, so overlapping calls each saw the session and each wrote a paid record. It is now serialized; the second caller gets null.</t>
+        </is>
+      </c>
+      <c r="G146" s="16" t="inlineStr">
+        <is>
+          <t>1.1.8</t>
+        </is>
+      </c>
+      <c r="H146" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="40" customHeight="1">
+      <c r="A147" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B147" s="16" t="inlineStr">
+        <is>
+          <t>56843dd</t>
+        </is>
+      </c>
+      <c r="C147" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D147" s="15" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="E147" s="18" t="inlineStr">
+        <is>
+          <t>An out-of-order EXPIRATION could revoke a renewed subscriber</t>
+        </is>
+      </c>
+      <c r="F147" s="18" t="inlineStr">
+        <is>
+          <t>The webhook only de-duplicated by event id, and RevenueCat can redeliver out of order. Writes now apply only if the event is at least as new as the last applied one (event_timestamp_ms vs rc_last_event_at, checked in the UPDATE). Also, the ledger row was written before the profile update, so a delivery that 500'd was dropped as a duplicate on retry; it is now written after. Deployed 2026-10-01.</t>
+        </is>
+      </c>
+      <c r="G147" s="16" t="inlineStr">
+        <is>
+          <t>1.1.8</t>
+        </is>
+      </c>
+      <c r="H147" s="22" t="inlineStr">
+        <is>
+          <t>Edge deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="40" customHeight="1">
+      <c r="A148" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B148" s="16" t="inlineStr">
+        <is>
+          <t>56843dd</t>
+        </is>
+      </c>
+      <c r="C148" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D148" s="15" t="inlineStr">
+        <is>
+          <t>Codes</t>
+        </is>
+      </c>
+      <c r="E148" s="18" t="inlineStr">
+        <is>
+          <t>A class redeeming a study code on one school network was blocked after 20</t>
+        </is>
+      </c>
+      <c r="F148" s="18" t="inlineStr">
+        <is>
+          <t>The per-IP hourly limit counted successful redemptions as attempts. It now counts failed guesses only, which is what brute force produces. Deployed 2026-10-01.</t>
+        </is>
+      </c>
+      <c r="G148" s="16" t="inlineStr">
+        <is>
+          <t>1.1.8</t>
+        </is>
+      </c>
+      <c r="H148" s="22" t="inlineStr">
+        <is>
+          <t>Edge deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="40" customHeight="1">
+      <c r="A149" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B149" s="16" t="inlineStr">
+        <is>
+          <t>56843dd</t>
+        </is>
+      </c>
+      <c r="C149" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D149" s="15" t="inlineStr">
+        <is>
+          <t>Screen Time</t>
+        </is>
+      </c>
+      <c r="E149" s="18" t="inlineStr">
+        <is>
+          <t>Background shield blocked every app category for non-Pro users</t>
+        </is>
+      </c>
+      <c r="F149" s="18" t="inlineStr">
+        <is>
+          <t>The DriftMonitor extension forced .all categories for any non-Pro user when the balance ran out, while the in-app path had already moved to honouring the user's picks. The extension now matches: picks win, and .all is only the fallback when nothing is picked.</t>
+        </is>
+      </c>
+      <c r="G149" s="16" t="inlineStr">
+        <is>
+          <t>1.1.8</t>
+        </is>
+      </c>
+      <c r="H149" s="22" t="inlineStr">
+        <is>
+          <t>Native build</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="40" customHeight="1">
+      <c r="A150" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B150" s="16" t="inlineStr">
+        <is>
+          <t>56843dd</t>
+        </is>
+      </c>
+      <c r="C150" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D150" s="15" t="inlineStr">
+        <is>
+          <t>Codes</t>
+        </is>
+      </c>
+      <c r="E150" s="18" t="inlineStr">
+        <is>
+          <t>Redeeming a dated code after a revoke restored permanent access</t>
+        </is>
+      </c>
+      <c r="F150" s="18" t="inlineStr">
+        <is>
+          <t>redeem_cohort_code's never-shorten rule treated a revoked grant (granted = false, expires_at null) as permanent, so any later 30-day code came back permanent with the old child seats. schema_v20 only honours an existing grant that is live. Migration written; not yet pushed.</t>
+        </is>
+      </c>
+      <c r="G150" s="16" t="inlineStr">
+        <is>
+          <t>1.1.8</t>
+        </is>
+      </c>
+      <c r="H150" s="22" t="inlineStr">
+        <is>
+          <t>SQL migration</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H145"/>
+  <autoFilter ref="A1:H150"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(changelog): 1.2.0 loyalty pricing
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Drift-changelog.xlsx
+++ b/Drift-changelog.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Changes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$158</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-10-11.</t>
+          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-10-12.</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Changes!E2:E157)</f>
+        <f>COUNTA(Changes!E2:E158)</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$157,A8)</f>
+        <f>COUNTIF(Changes!$C$2:$C$158,A8)</f>
         <v/>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D8)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D8)</f>
         <v/>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$157,G8)</f>
+        <f>COUNTIF(Changes!$G$2:$G$158,G8)</f>
         <v/>
       </c>
     </row>
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$157,A9)</f>
+        <f>COUNTIF(Changes!$C$2:$C$158,A9)</f>
         <v/>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D9)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D9)</f>
         <v/>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$157,G9)</f>
+        <f>COUNTIF(Changes!$G$2:$G$158,G9)</f>
         <v/>
       </c>
     </row>
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$157,A10)</f>
+        <f>COUNTIF(Changes!$C$2:$C$158,A10)</f>
         <v/>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D10)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D10)</f>
         <v/>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$157,G10)</f>
+        <f>COUNTIF(Changes!$G$2:$G$158,G10)</f>
         <v/>
       </c>
     </row>
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$157,A11)</f>
+        <f>COUNTIF(Changes!$C$2:$C$158,A11)</f>
         <v/>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D11)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D11)</f>
         <v/>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$157,G11)</f>
+        <f>COUNTIF(Changes!$G$2:$G$158,G11)</f>
         <v/>
       </c>
     </row>
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$157,A12)</f>
+        <f>COUNTIF(Changes!$C$2:$C$158,A12)</f>
         <v/>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D12)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D12)</f>
         <v/>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="H12" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$157,G12)</f>
+        <f>COUNTIF(Changes!$G$2:$G$158,G12)</f>
         <v/>
       </c>
     </row>
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$157,A13)</f>
+        <f>COUNTIF(Changes!$C$2:$C$158,A13)</f>
         <v/>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="E13" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D13)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D13)</f>
         <v/>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="H13" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$157,G13)</f>
+        <f>COUNTIF(Changes!$G$2:$G$158,G13)</f>
         <v/>
       </c>
     </row>
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$157,A14)</f>
+        <f>COUNTIF(Changes!$C$2:$C$158,A14)</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="E14" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D14)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D14)</f>
         <v/>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="H14" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$157,G14)</f>
+        <f>COUNTIF(Changes!$G$2:$G$158,G14)</f>
         <v/>
       </c>
     </row>
@@ -852,7 +852,7 @@
         </is>
       </c>
       <c r="E15" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D15)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D15)</f>
         <v/>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="H15" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$157,G15)</f>
+        <f>COUNTIF(Changes!$G$2:$G$158,G15)</f>
         <v/>
       </c>
     </row>
@@ -872,7 +872,7 @@
         </is>
       </c>
       <c r="E16" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D16)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D16)</f>
         <v/>
       </c>
     </row>
@@ -883,7 +883,7 @@
         </is>
       </c>
       <c r="E17" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D17)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D17)</f>
         <v/>
       </c>
     </row>
@@ -894,7 +894,7 @@
         </is>
       </c>
       <c r="E18" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D18)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D18)</f>
         <v/>
       </c>
     </row>
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="E19" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D19)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D19)</f>
         <v/>
       </c>
     </row>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="E20" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D20)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D20)</f>
         <v/>
       </c>
     </row>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="E21" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D21)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D21)</f>
         <v/>
       </c>
     </row>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="E22" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D22)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D22)</f>
         <v/>
       </c>
     </row>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="E23" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D23)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D23)</f>
         <v/>
       </c>
     </row>
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="E24" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D24)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D24)</f>
         <v/>
       </c>
     </row>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="E25" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D25)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D25)</f>
         <v/>
       </c>
     </row>
@@ -982,7 +982,7 @@
         </is>
       </c>
       <c r="E26" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D26)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D26)</f>
         <v/>
       </c>
     </row>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="E27" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D27)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D27)</f>
         <v/>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="E28" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D28)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D28)</f>
         <v/>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="E29" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D29)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D29)</f>
         <v/>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
         </is>
       </c>
       <c r="E30" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D30)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D30)</f>
         <v/>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="E31" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D31)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D31)</f>
         <v/>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
         </is>
       </c>
       <c r="E32" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D32)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D32)</f>
         <v/>
       </c>
     </row>
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="E33" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D33)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D33)</f>
         <v/>
       </c>
     </row>
@@ -1070,7 +1070,7 @@
         </is>
       </c>
       <c r="E34" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D34)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D34)</f>
         <v/>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
         </is>
       </c>
       <c r="E35" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D35)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D35)</f>
         <v/>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="E36" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D36)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D36)</f>
         <v/>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="E37" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D37)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D37)</f>
         <v/>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="E38" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D38)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D38)</f>
         <v/>
       </c>
     </row>
@@ -1125,7 +1125,7 @@
         </is>
       </c>
       <c r="E39" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D39)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D39)</f>
         <v/>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
         </is>
       </c>
       <c r="E40" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D40)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D40)</f>
         <v/>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="E41" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D41)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D41)</f>
         <v/>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
         </is>
       </c>
       <c r="E42" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D42)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D42)</f>
         <v/>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="E43" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D43)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D43)</f>
         <v/>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="E44" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D44)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D44)</f>
         <v/>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="E45" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D45)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D45)</f>
         <v/>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
         </is>
       </c>
       <c r="E46" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D46)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D46)</f>
         <v/>
       </c>
     </row>
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="E47" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D47)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D47)</f>
         <v/>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="E48" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D48)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D48)</f>
         <v/>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="E49" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D49)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D49)</f>
         <v/>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="E50" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D50)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D50)</f>
         <v/>
       </c>
     </row>
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="E51" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D51)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D51)</f>
         <v/>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
         </is>
       </c>
       <c r="E52" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D52)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D52)</f>
         <v/>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
         </is>
       </c>
       <c r="E53" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$157,D53)</f>
+        <f>COUNTIF(Changes!$D$2:$D$158,D53)</f>
         <v/>
       </c>
     </row>
@@ -1329,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H157"/>
+  <dimension ref="A1:H158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7928,8 +7928,50 @@
         </is>
       </c>
     </row>
+    <row r="158" ht="40" customHeight="1">
+      <c r="A158" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B158" s="16" t="inlineStr">
+        <is>
+          <t>90dc57e</t>
+        </is>
+      </c>
+      <c r="C158" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D158" s="15" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+      <c r="E158" s="18" t="inlineStr">
+        <is>
+          <t>Loyalty pricing: monthly Pro drops 50¢ every 2 months, down to $2.99</t>
+        </is>
+      </c>
+      <c r="F158" s="18" t="inlineStr">
+        <is>
+          <t>$4.99 for months 0-1, then $4.49, $3.99, $3.49 and $2.99 from month 8, counted over an unbroken paid run (trial days excluded). Unsubscribing or lapsing resets it. Apple won't let an app change one subscriber's price, so each step is a promotional offer on com.drift.pro.month (loyalty_449/399/349 for 2 months, loyalty_299 for 12) that the subscriber confirms once; it starts at their next renewal. The webhook keeps profiles.sub_paid_since (guarded like the other subscription columns). Ships switched off: needs schema_v22 pushed, the webhook deployed, the four offers in App Store Connect, the subscription key in RevenueCat, then app_config.loyalty_pricing = 'true'.</t>
+        </is>
+      </c>
+      <c r="G158" s="16" t="inlineStr">
+        <is>
+          <t>1.2.0</t>
+        </is>
+      </c>
+      <c r="H158" s="22" t="inlineStr">
+        <is>
+          <t>SQL migration, Edge deploy, App Store Connect</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H157"/>
+  <autoFilter ref="A1:H158"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(changelog): 1.2.0 simpler paywall
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Drift-changelog.xlsx
+++ b/Drift-changelog.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Changes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$158</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$159</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Changes!E2:E158)</f>
+        <f>COUNTA(Changes!E2:E159)</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$158,A8)</f>
+        <f>COUNTIF(Changes!$C$2:$C$159,A8)</f>
         <v/>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D8)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D8)</f>
         <v/>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$158,G8)</f>
+        <f>COUNTIF(Changes!$G$2:$G$159,G8)</f>
         <v/>
       </c>
     </row>
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$158,A9)</f>
+        <f>COUNTIF(Changes!$C$2:$C$159,A9)</f>
         <v/>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D9)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D9)</f>
         <v/>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$158,G9)</f>
+        <f>COUNTIF(Changes!$G$2:$G$159,G9)</f>
         <v/>
       </c>
     </row>
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$158,A10)</f>
+        <f>COUNTIF(Changes!$C$2:$C$159,A10)</f>
         <v/>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D10)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D10)</f>
         <v/>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$158,G10)</f>
+        <f>COUNTIF(Changes!$G$2:$G$159,G10)</f>
         <v/>
       </c>
     </row>
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$158,A11)</f>
+        <f>COUNTIF(Changes!$C$2:$C$159,A11)</f>
         <v/>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D11)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D11)</f>
         <v/>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$158,G11)</f>
+        <f>COUNTIF(Changes!$G$2:$G$159,G11)</f>
         <v/>
       </c>
     </row>
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$158,A12)</f>
+        <f>COUNTIF(Changes!$C$2:$C$159,A12)</f>
         <v/>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D12)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D12)</f>
         <v/>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="H12" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$158,G12)</f>
+        <f>COUNTIF(Changes!$G$2:$G$159,G12)</f>
         <v/>
       </c>
     </row>
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$158,A13)</f>
+        <f>COUNTIF(Changes!$C$2:$C$159,A13)</f>
         <v/>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="E13" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D13)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D13)</f>
         <v/>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="H13" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$158,G13)</f>
+        <f>COUNTIF(Changes!$G$2:$G$159,G13)</f>
         <v/>
       </c>
     </row>
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$158,A14)</f>
+        <f>COUNTIF(Changes!$C$2:$C$159,A14)</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="E14" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D14)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D14)</f>
         <v/>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="H14" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$158,G14)</f>
+        <f>COUNTIF(Changes!$G$2:$G$159,G14)</f>
         <v/>
       </c>
     </row>
@@ -852,7 +852,7 @@
         </is>
       </c>
       <c r="E15" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D15)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D15)</f>
         <v/>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="H15" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$158,G15)</f>
+        <f>COUNTIF(Changes!$G$2:$G$159,G15)</f>
         <v/>
       </c>
     </row>
@@ -872,7 +872,7 @@
         </is>
       </c>
       <c r="E16" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D16)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D16)</f>
         <v/>
       </c>
     </row>
@@ -883,7 +883,7 @@
         </is>
       </c>
       <c r="E17" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D17)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D17)</f>
         <v/>
       </c>
     </row>
@@ -894,7 +894,7 @@
         </is>
       </c>
       <c r="E18" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D18)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D18)</f>
         <v/>
       </c>
     </row>
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="E19" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D19)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D19)</f>
         <v/>
       </c>
     </row>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="E20" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D20)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D20)</f>
         <v/>
       </c>
     </row>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="E21" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D21)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D21)</f>
         <v/>
       </c>
     </row>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="E22" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D22)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D22)</f>
         <v/>
       </c>
     </row>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="E23" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D23)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D23)</f>
         <v/>
       </c>
     </row>
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="E24" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D24)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D24)</f>
         <v/>
       </c>
     </row>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="E25" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D25)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D25)</f>
         <v/>
       </c>
     </row>
@@ -982,7 +982,7 @@
         </is>
       </c>
       <c r="E26" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D26)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D26)</f>
         <v/>
       </c>
     </row>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="E27" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D27)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D27)</f>
         <v/>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="E28" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D28)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D28)</f>
         <v/>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="E29" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D29)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D29)</f>
         <v/>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
         </is>
       </c>
       <c r="E30" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D30)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D30)</f>
         <v/>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="E31" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D31)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D31)</f>
         <v/>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
         </is>
       </c>
       <c r="E32" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D32)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D32)</f>
         <v/>
       </c>
     </row>
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="E33" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D33)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D33)</f>
         <v/>
       </c>
     </row>
@@ -1070,7 +1070,7 @@
         </is>
       </c>
       <c r="E34" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D34)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D34)</f>
         <v/>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
         </is>
       </c>
       <c r="E35" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D35)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D35)</f>
         <v/>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="E36" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D36)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D36)</f>
         <v/>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="E37" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D37)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D37)</f>
         <v/>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="E38" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D38)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D38)</f>
         <v/>
       </c>
     </row>
@@ -1125,7 +1125,7 @@
         </is>
       </c>
       <c r="E39" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D39)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D39)</f>
         <v/>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
         </is>
       </c>
       <c r="E40" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D40)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D40)</f>
         <v/>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="E41" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D41)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D41)</f>
         <v/>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
         </is>
       </c>
       <c r="E42" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D42)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D42)</f>
         <v/>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="E43" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D43)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D43)</f>
         <v/>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="E44" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D44)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D44)</f>
         <v/>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="E45" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D45)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D45)</f>
         <v/>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
         </is>
       </c>
       <c r="E46" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D46)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D46)</f>
         <v/>
       </c>
     </row>
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="E47" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D47)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D47)</f>
         <v/>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="E48" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D48)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D48)</f>
         <v/>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="E49" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D49)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D49)</f>
         <v/>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="E50" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D50)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D50)</f>
         <v/>
       </c>
     </row>
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="E51" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D51)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D51)</f>
         <v/>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
         </is>
       </c>
       <c r="E52" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D52)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D52)</f>
         <v/>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
         </is>
       </c>
       <c r="E53" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$158,D53)</f>
+        <f>COUNTIF(Changes!$D$2:$D$159,D53)</f>
         <v/>
       </c>
     </row>
@@ -1329,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H158"/>
+  <dimension ref="A1:H159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7970,8 +7970,50 @@
         </is>
       </c>
     </row>
+    <row r="159" ht="40" customHeight="1">
+      <c r="A159" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B159" s="16" t="inlineStr">
+        <is>
+          <t>36aef9e</t>
+        </is>
+      </c>
+      <c r="C159" s="23" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D159" s="15" t="inlineStr">
+        <is>
+          <t>Paywall</t>
+        </is>
+      </c>
+      <c r="E159" s="18" t="inlineStr">
+        <is>
+          <t>Simpler Pro sheet, and it shows loyalty pricing</t>
+        </is>
+      </c>
+      <c r="F159" s="18" t="inlineStr">
+        <is>
+          <t>Down to a name, one line on what Pro adds, two plan rows and one button (trial on the button), from a two-line headline, four bullets and tiles. Monthly reads 'Your price drops every 2 months you stay, down to $2.99/mo' using Apple's localized floor price, only while loyalty_pricing is on and the offer exists; the terms add that each lower price is offered in the app to accept. Apple 3.1.2 items unchanged.</t>
+        </is>
+      </c>
+      <c r="G159" s="16" t="inlineStr">
+        <is>
+          <t>1.2.0</t>
+        </is>
+      </c>
+      <c r="H159" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H158"/>
+  <autoFilter ref="A1:H159"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(release): 1.3.0 — languages and children's privacy
Version bumped in app.json, package.json and MARKETING_VERSION.
Changelog rows for the i18n and COPPA work.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Drift-changelog.xlsx
+++ b/Drift-changelog.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Changes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$159</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes'!$A$1:$H$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -578,7 +578,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-10-12.</t>
+          <t>Every feature, fix and change shipped. 2026-07-07 – 2026-10-26.</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTA(Changes!E2:E159)</f>
+        <f>COUNTA(Changes!E2:E164)</f>
         <v/>
       </c>
     </row>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$159,A8)</f>
+        <f>COUNTIF(Changes!$C$2:$C$164,A8)</f>
         <v/>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D8)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D8)</f>
         <v/>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="H8" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$159,G8)</f>
+        <f>COUNTIF(Changes!$G$2:$G$164,G8)</f>
         <v/>
       </c>
     </row>
@@ -678,16 +678,16 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$159,A9)</f>
+        <f>COUNTIF(Changes!$C$2:$C$164,A9)</f>
         <v/>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Action Plan</t>
+          <t>Account</t>
         </is>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D9)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D9)</f>
         <v/>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="H9" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$159,G9)</f>
+        <f>COUNTIF(Changes!$G$2:$G$164,G9)</f>
         <v/>
       </c>
     </row>
@@ -707,16 +707,16 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$159,A10)</f>
+        <f>COUNTIF(Changes!$C$2:$C$164,A10)</f>
         <v/>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Add Task</t>
+          <t>Action Plan</t>
         </is>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D10)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D10)</f>
         <v/>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="H10" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$159,G10)</f>
+        <f>COUNTIF(Changes!$G$2:$G$164,G10)</f>
         <v/>
       </c>
     </row>
@@ -736,16 +736,16 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$159,A11)</f>
+        <f>COUNTIF(Changes!$C$2:$C$164,A11)</f>
         <v/>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Analytics</t>
+          <t>Add Task</t>
         </is>
       </c>
       <c r="E11" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D11)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D11)</f>
         <v/>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="H11" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$159,G11)</f>
+        <f>COUNTIF(Changes!$G$2:$G$164,G11)</f>
         <v/>
       </c>
     </row>
@@ -765,16 +765,16 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$159,A12)</f>
+        <f>COUNTIF(Changes!$C$2:$C$164,A12)</f>
         <v/>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Auth</t>
+          <t>Analytics</t>
         </is>
       </c>
       <c r="E12" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D12)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D12)</f>
         <v/>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="H12" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$159,G12)</f>
+        <f>COUNTIF(Changes!$G$2:$G$164,G12)</f>
         <v/>
       </c>
     </row>
@@ -794,16 +794,16 @@
         </is>
       </c>
       <c r="B13" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$159,A13)</f>
+        <f>COUNTIF(Changes!$C$2:$C$164,A13)</f>
         <v/>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Auth / Sync</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="E13" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D13)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D13)</f>
         <v/>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="H13" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$159,G13)</f>
+        <f>COUNTIF(Changes!$G$2:$G$164,G13)</f>
         <v/>
       </c>
     </row>
@@ -823,16 +823,16 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>COUNTIF(Changes!$C$2:$C$159,A14)</f>
+        <f>COUNTIF(Changes!$C$2:$C$164,A14)</f>
         <v/>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Backend</t>
+          <t>Auth / Sync</t>
         </is>
       </c>
       <c r="E14" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D14)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D14)</f>
         <v/>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -841,478 +841,513 @@
         </is>
       </c>
       <c r="H14" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$159,G14)</f>
+        <f>COUNTIF(Changes!$G$2:$G$164,G14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Billing</t>
+          <t>Backend</t>
         </is>
       </c>
       <c r="E15" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D15)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D15)</f>
         <v/>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Unreleased</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="H15" s="7">
-        <f>COUNTIF(Changes!$G$2:$G$159,G15)</f>
+        <f>COUNTIF(Changes!$G$2:$G$164,G15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>CI/CD</t>
+          <t>Billing</t>
         </is>
       </c>
       <c r="E16" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D16)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D16)</f>
+        <v/>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="H16" s="7">
+        <f>COUNTIF(Changes!$G$2:$G$164,G16)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>CI/CD</t>
         </is>
       </c>
       <c r="E17" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D17)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Challenges</t>
+          <t>Calendar</t>
         </is>
       </c>
       <c r="E18" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D18)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Codes</t>
+          <t>Challenges</t>
         </is>
       </c>
       <c r="E19" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D19)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Cohort codes</t>
+          <t>Codes</t>
         </is>
       </c>
       <c r="E20" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D20)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Dependencies</t>
+          <t>Cohort codes</t>
         </is>
       </c>
       <c r="E21" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D21)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D21)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Dev</t>
+          <t>Dependencies</t>
         </is>
       </c>
       <c r="E22" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D22)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D22)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Discoverability</t>
+          <t>Dev</t>
         </is>
       </c>
       <c r="E23" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D23)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D23)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Drift In</t>
+          <t>Discoverability</t>
         </is>
       </c>
       <c r="E24" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D24)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D24)</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>Drift In</t>
         </is>
       </c>
       <c r="E25" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D25)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>Entitlement</t>
         </is>
       </c>
       <c r="E26" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D26)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Force update</t>
+          <t>Family</t>
         </is>
       </c>
       <c r="E27" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D27)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Growth</t>
+          <t>Force update</t>
         </is>
       </c>
       <c r="E28" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D28)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D28)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Interaction</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="E29" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D29)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D29)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Lab</t>
+          <t>Interaction</t>
         </is>
       </c>
       <c r="E30" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D30)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D30)</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Live Activity</t>
+          <t>Lab</t>
         </is>
       </c>
       <c r="E31" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D31)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D31)</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Lockbox</t>
+          <t>Live Activity</t>
         </is>
       </c>
       <c r="E32" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D32)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D32)</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Lockbox</t>
         </is>
       </c>
       <c r="E33" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D33)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D33)</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="E34" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D34)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D34)</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E35" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D35)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D35)</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="E36" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D36)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D36)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Paywall</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="E37" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D37)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D37)</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Paywall</t>
         </is>
       </c>
       <c r="E38" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D38)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D38)</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E39" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D39)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D39)</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Privacy</t>
         </is>
       </c>
       <c r="E40" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D40)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D40)</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="E41" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D41)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D41)</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Reviews</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="E42" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D42)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D42)</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Scaling</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="E43" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D43)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D43)</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Screen Time</t>
+          <t>Reviews</t>
         </is>
       </c>
       <c r="E44" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D44)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D44)</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Shield</t>
+          <t>Scaling</t>
         </is>
       </c>
       <c r="E45" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D45)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D45)</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Siri</t>
+          <t>Screen Time</t>
         </is>
       </c>
       <c r="E46" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D46)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D46)</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Sleep Guard</t>
+          <t>Shield</t>
         </is>
       </c>
       <c r="E47" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D47)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D47)</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Social</t>
+          <t>Siri</t>
         </is>
       </c>
       <c r="E48" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D48)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D48)</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Tasks</t>
+          <t>Sleep Guard</t>
         </is>
       </c>
       <c r="E49" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D49)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D49)</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>Social</t>
         </is>
       </c>
       <c r="E50" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D50)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D50)</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Tour</t>
+          <t>Tasks</t>
         </is>
       </c>
       <c r="E51" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D51)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D51)</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Theme</t>
         </is>
       </c>
       <c r="E52" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D52)</f>
+        <f>COUNTIF(Changes!$D$2:$D$164,D52)</f>
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="D53" s="7" t="inlineStr">
         <is>
+          <t>Tour</t>
+        </is>
+      </c>
+      <c r="E53" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$164,D53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="E54" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$164,D54)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="D55" s="7" t="inlineStr">
+        <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="E53" s="7">
-        <f>COUNTIF(Changes!$D$2:$D$159,D53)</f>
+      <c r="E55" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$164,D55)</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>i18n</t>
+        </is>
+      </c>
+      <c r="E56" s="7">
+        <f>COUNTIF(Changes!$D$2:$D$164,D56)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="13" t="inlineStr">
-        <is>
-          <t>• 1.1.8 is the last version submitted to the App Store. Everything marked Unreleased is on main but not shipped.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="13" t="inlineStr">
-        <is>
-          <t>• "Needs" says what a change requires beyond a normal JS reload: a native rebuild, an edge-function deploy, or SQL run in Supabase.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="13" t="inlineStr">
-        <is>
-          <t>• Native-build items are currently blocked on Apple Developer account access, so they are not device-tested.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>• 1.2.0 is the version live on the App Store; 1.3.0 is the next submission. Everything marked Unreleased is on main but not shipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>• "Needs" says what a change requires beyond a normal JS reload: a native rebuild, an edge-function deploy, or SQL run in Supabase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
         <is>
           <t>• Counts on this sheet are formulas over the Changes tab — they update if you edit, add or delete rows there.</t>
         </is>
@@ -1329,7 +1364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H159"/>
+  <dimension ref="A1:H164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8012,8 +8047,218 @@
         </is>
       </c>
     </row>
+    <row r="160" ht="40" customHeight="1">
+      <c r="A160" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B160" s="16" t="inlineStr">
+        <is>
+          <t>cf38bc0</t>
+        </is>
+      </c>
+      <c r="C160" s="17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D160" s="15" t="inlineStr">
+        <is>
+          <t>i18n</t>
+        </is>
+      </c>
+      <c r="E160" s="18" t="inlineStr">
+        <is>
+          <t>App available in 20 languages</t>
+        </is>
+      </c>
+      <c r="F160" s="18" t="inlineStr">
+        <is>
+          <t>English plus Simplified/Traditional Chinese, Hindi, Spanish, French, Arabic, Portuguese, Russian, Indonesian, German, Japanese, Turkish, Vietnamese, Korean, Italian, Polish, Ukrainian, Thai and Dutch. English-as-key tr() with lazy-loaded catalogs; follows the device language or a picker in Profile (switching reloads the JS). Push notifications, AI feedback, the Screen Time shield/widgets and iOS permission prompts are translated too. Machine-authored translations, not reviewed by native speakers. Arabic text is translated but the layout is not mirrored.</t>
+        </is>
+      </c>
+      <c r="G160" s="16" t="inlineStr">
+        <is>
+          <t>1.3.0</t>
+        </is>
+      </c>
+      <c r="H160" s="22" t="inlineStr">
+        <is>
+          <t>Native build, Edge deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="40" customHeight="1">
+      <c r="A161" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B161" s="16" t="inlineStr">
+        <is>
+          <t>cf38bc0</t>
+        </is>
+      </c>
+      <c r="C161" s="24" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="D161" s="15" t="inlineStr">
+        <is>
+          <t>Privacy</t>
+        </is>
+      </c>
+      <c r="E161" s="18" t="inlineStr">
+        <is>
+          <t>Parental consent before a child can join a family</t>
+        </is>
+      </c>
+      <c r="F161" s="18" t="inlineStr">
+        <is>
+          <t>COPPA needs verifiable parental consent before collecting data from under-13s. Parents now see a direct notice (what is collected, who sees it, retention, rights) and consent; the Drift Family purchase is the verification method. join-family refuses a code until the family has consented (deploy join-family only once 1.3.0 is live, or current-version families can't add children). Parents can view, delete per child, or withdraw consent (erases every child). Consent is versioned and logged in parental_consent_events.</t>
+        </is>
+      </c>
+      <c r="G161" s="16" t="inlineStr">
+        <is>
+          <t>1.3.0</t>
+        </is>
+      </c>
+      <c r="H161" s="22" t="inlineStr">
+        <is>
+          <t>SQL migration, Edge deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="40" customHeight="1">
+      <c r="A162" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B162" s="16" t="inlineStr">
+        <is>
+          <t>cf38bc0</t>
+        </is>
+      </c>
+      <c r="C162" s="19" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="D162" s="15" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="E162" s="18" t="inlineStr">
+        <is>
+          <t>Deleting an account left most of its data behind</t>
+        </is>
+      </c>
+      <c r="F162" s="18" t="inlineStr">
+        <is>
+          <t>delete-account called .delete() on tables guarded by prevent_hard_delete(), which raised, and the errors were swallowed, so tasks, ledger, analytics etc. survived. erase_account() (service-role only) now erases every user table under a transaction-local drift.erasure flag, scrubs the profile, and erases a parent's children too. Also revokes the Sign in with Apple token (Apple requires it; needs the APPLE_* secrets). Migration applied 2026-10-26 and verified live.</t>
+        </is>
+      </c>
+      <c r="G162" s="16" t="inlineStr">
+        <is>
+          <t>1.3.0</t>
+        </is>
+      </c>
+      <c r="H162" s="22" t="inlineStr">
+        <is>
+          <t>SQL migration, Edge deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="40" customHeight="1">
+      <c r="A163" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B163" s="16" t="inlineStr">
+        <is>
+          <t>cf38bc0</t>
+        </is>
+      </c>
+      <c r="C163" s="24" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="D163" s="15" t="inlineStr">
+        <is>
+          <t>Privacy</t>
+        </is>
+      </c>
+      <c r="E163" s="18" t="inlineStr">
+        <is>
+          <t>Children kept out of AI checks and analytics; retention purge</t>
+        </is>
+      </c>
+      <c r="F163" s="18" t="inlineStr">
+        <is>
+          <t>verify-task and evaluate-task reject child accounts, so nothing a child does reaches OpenAI; child analytics are disabled client-side, refused by RLS, and existing rows deleted. purge_expired_data() runs nightly via pg_cron (analytics 13 months, AI usage 90 days, push tokens 9 months, inactive child accounts 18 months). Neutral age gate at sign-up: 13+ for personal, 18+ for parent.</t>
+        </is>
+      </c>
+      <c r="G163" s="16" t="inlineStr">
+        <is>
+          <t>1.3.0</t>
+        </is>
+      </c>
+      <c r="H163" s="22" t="inlineStr">
+        <is>
+          <t>SQL migration, Edge deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="40" customHeight="1">
+      <c r="A164" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B164" s="16" t="inlineStr">
+        <is>
+          <t>cf38bc0</t>
+        </is>
+      </c>
+      <c r="C164" s="21" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D164" s="15" t="inlineStr">
+        <is>
+          <t>Privacy</t>
+        </is>
+      </c>
+      <c r="E164" s="18" t="inlineStr">
+        <is>
+          <t>Privacy policy rewritten to match what the app does</t>
+        </is>
+      </c>
+      <c r="F164" s="18" t="inlineStr">
+        <is>
+          <t>The old policy omitted data the app collects and named a processor it no longer uses. New one lists every data type and provider, a children's section, a retention table, CCPA/GDPR/consumer-health-data rights. Plus SECURITY_PROGRAM.md (the written security program COPPA requires).</t>
+        </is>
+      </c>
+      <c r="G164" s="16" t="inlineStr">
+        <is>
+          <t>1.3.0</t>
+        </is>
+      </c>
+      <c r="H164" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H159"/>
+  <autoFilter ref="A1:H164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>